<commit_message>
cicada IG: refresh the site copy from today's 0-error build
Built with publisher 2.3.4 from cicada 4fca0a89, 2026-09-06, 2 min 32 s,
0 errors, 411 warnings. The previous copy (632d4887) predated the logical
models, the StructureMap corrections, the ICD-10-CM stub, the SNOMED US
edition, the regenerated maps and the regenerated forecast example.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014oU3PKgtLkXXkkKZoLLRok
</commit_message>
<xml_diff>
--- a/jaspr/web/cicada_ig/StructureDefinition-Vaccine.xlsx
+++ b/jaspr/web/cicada_ig/StructureDefinition-Vaccine.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://example.org/fhir/StructureDefinition/Vaccine</t>
+    <t>http://fhirfli.dev/fhir/ig/cicada/StructureDefinition/Vaccine</t>
   </si>
   <si>
     <t>Version</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-02T22:18:14-04:00</t>
+    <t>2026-09-06T20:44:07-04:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>